<commit_message>
Batch content updates from spreadsheet: reorder values (D/El/Em/C), remove LogoTicker, foundation→charity number, media logos removed, TikTok→LinkedIn, navbar updated (Events added, Foundation/Media removed, Contact→#contact), SPN initiative added, insight tabs→4 values, team subtitle updated, events page created, team page values→DEEC, 8→9 initiatives count, heading→Creating Lasting Impact
</commit_message>
<xml_diff>
--- a/Devanhaar Website.xlsx
+++ b/Devanhaar Website.xlsx
@@ -5,8 +5,10 @@
   <sheets>
     <sheet state="visible" name="Home" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="About " sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Initiatives " sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Other" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="Donate" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Team " sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="Initiatives " sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Other" sheetId="6" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -14,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="136">
   <si>
     <t xml:space="preserve">Old </t>
   </si>
@@ -46,7 +48,7 @@
     <t xml:space="preserve">Built by a team from </t>
   </si>
   <si>
-    <t xml:space="preserve">Do we put in all the organisations we work with? </t>
+    <t xml:space="preserve">Remove all of this </t>
   </si>
   <si>
     <t xml:space="preserve">DEVELOP </t>
@@ -148,6 +150,187 @@
     <t xml:space="preserve">1000+ Campers </t>
   </si>
   <si>
+    <t xml:space="preserve">On homepage, remove the section where it says our mission </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove all the cards - go straight from our pillars to our initiatives </t>
+  </si>
+  <si>
+    <t>Change fuirst word order</t>
+  </si>
+  <si>
+    <t>Develop. Elevate. Empower. Connect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make empower the word in colour - thats the main </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensure this order is reflected in our pillars. Make empower the orangey colour </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep this </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under key initiatives make four cards </t>
+  </si>
+  <si>
+    <t>card under Develop</t>
+  </si>
+  <si>
+    <t>Photo of someone delivering a talk. Put a figure underneath, 1000+ hours of workshops delivered across all of our organisations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">card under elevate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photo of khalsa catalyst (show a kid being elevated). 20,000+ Futures Supported </t>
+  </si>
+  <si>
+    <t>Card under empower</t>
+  </si>
+  <si>
+    <t>photo of muy thai academy, show something about strength. 400+ Youth Empowered</t>
+  </si>
+  <si>
+    <t>card under connect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two people laughing . 50+ events anually </t>
+  </si>
+  <si>
+    <t xml:space="preserve">All insights </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change education, community, leadership to our four values </t>
+  </si>
+  <si>
+    <t>Meet the People Behind</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Underneath this put </t>
+  </si>
+  <si>
+    <t>the Mission</t>
+  </si>
+  <si>
+    <t>Passionate individuals committed to empowering and supporting the next generation.</t>
+  </si>
+  <si>
+    <t>Mandeep Narwal / head of operations</t>
+  </si>
+  <si>
+    <t>Take photo from linkedin and put in a small linkedin logo that is pressable and goes to their linkedin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baldev Singh/ Head of communication </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jitarun Singh, ACCA (take from linkedin)  / Account Lead </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daljit Kaur / Project Manager </t>
+  </si>
+  <si>
+    <t>Mandeep Singh / Joint Head of Finance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gugandeep Singh / Joint Head of Finance </t>
+  </si>
+  <si>
+    <t>Gurvinder Singh/ Head of HR &amp; Governance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bapinder Singh / Tech Manager </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inderjit Singh / Head of Self Defence Academy </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amrit Singh / Creative Lead </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gursimran Kaur / Head of Kaurs Camp </t>
+  </si>
+  <si>
+    <t>Benita / Head of Kaurs Spaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head of Media / Gurpreet Rana </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head of Singhs Camp / Pritam Singh </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head of Operations / Dr Taran Singh </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head of Partnerships / Sat Singh </t>
+  </si>
+  <si>
+    <t>Devanhaar Foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove and change to "Charity number: 1203393"
+</t>
+  </si>
+  <si>
+    <t>News / featured in media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Put a live pull of our recent instagram posts  </t>
+  </si>
+  <si>
+    <t>Remove these</t>
+  </si>
+  <si>
+    <t>SikhNetSikh Press AssociationBasics of SikhiSikh2InspireAsian ImageThe Sikh MessengerSikh ChannelPunjab2000</t>
+  </si>
+  <si>
+    <t>Footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove tiktok </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add linkedin (make one if we dont have one already) </t>
+  </si>
+  <si>
+    <t>DevnahaAR Initiatives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Also add sikh professional network (and this will then need to be under initiatives/ have its own page) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove the foundation tab - not needed </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove media from the tab </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add in a new tab called events </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navjot, i want this events tab to be where we promote yearly events like yorkshire 3 peaks, wolf run, and so forth </t>
+  </si>
+  <si>
+    <t>Example: Engagement
+Yorkshire 3 Peaks Hike - 27th June 2026
+Singhs Camp Wolf Run - 12th Sept 2026
+Paintballing - 30th Jan 2027
+Skills/Life
+Shooting - Weekly Course (£250/Year) 
+Bushcraft Training - (May/June)
+Wild Camping - (May/June)
+Horse Riding &amp; Seva (March onwards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact tab </t>
+  </si>
+  <si>
+    <t xml:space="preserve">This doesnt need to be a separate page. When pressed from homepage, have it scroll to the bottom section where it says Have a question or want to get involved?
+</t>
+  </si>
+  <si>
     <t>Old</t>
   </si>
   <si>
@@ -216,6 +399,52 @@
     <t xml:space="preserve">30+ events anually </t>
   </si>
   <si>
+    <t>Projects That Create Lasting Impact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change to "Creating lasting impact" </t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>Make all the cards the same size and add in SPN</t>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">This needs to link in with different payment methods (paypal, go cardless, stripe) - and then, this needs to link with </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>donationmanager.co.uk</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Our values </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change this to our devanhaar values </t>
+  </si>
+  <si>
+    <t>Join Our Sevadaar Family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Join our team </t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove location, put UK </t>
+  </si>
+  <si>
+    <t>Birmingham, United Kingdom</t>
+  </si>
+  <si>
     <t>Change tab. - projects to initiatives</t>
   </si>
   <si>
@@ -235,7 +464,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="15">
+  <fonts count="20">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -301,11 +530,30 @@
       <name val="Ui-sans-serif"/>
     </font>
     <font>
+      <sz val="12.0"/>
+      <color rgb="FF22252A"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF946A00"/>
+      <name val="Ui-sans-serif"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
+      <color rgb="FF946A00"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12.0"/>
+      <color rgb="FF6D7178"/>
+      <name val="Ui-sans-serif"/>
+    </font>
+    <font>
       <u/>
       <color rgb="FF0000FF"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
       <color rgb="FF22252A"/>
       <name val="Arial"/>
     </font>
@@ -313,13 +561,23 @@
       <color rgb="FF6D7178"/>
       <name val="Ui-sans-serif"/>
     </font>
+    <font>
+      <color rgb="FF22252A"/>
+      <name val="Ui-sans-serif"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -345,6 +603,12 @@
         <bgColor rgb="FFEBEDEF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A1F2E"/>
+        <bgColor rgb="FF1A1F2E"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -352,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -368,41 +632,71 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="11" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="6" fontId="11" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="6" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -426,6 +720,14 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -634,8 +936,8 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="40.38"/>
-    <col customWidth="1" min="2" max="2" width="92.13"/>
+    <col customWidth="1" min="1" max="1" width="53.75"/>
+    <col customWidth="1" min="2" max="2" width="114.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -769,10 +1071,10 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="2"/>
@@ -801,7 +1103,7 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -833,10 +1135,10 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="2"/>
@@ -865,10 +1167,10 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="2"/>
@@ -897,10 +1199,10 @@
       <c r="Z8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="2"/>
@@ -929,7 +1231,7 @@
       <c r="Z9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -961,7 +1263,7 @@
       <c r="Z10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1345,7 +1647,7 @@
       <c r="Z22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="13" t="s">
         <v>40</v>
       </c>
       <c r="B23" s="4" t="s">
@@ -1377,7 +1679,7 @@
       <c r="Z23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="14" t="s">
         <v>42</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -1409,7 +1711,7 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="14"/>
+      <c r="A25" s="15"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1437,8 +1739,12 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
+      <c r="A26" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -1465,10 +1771,18 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="A27" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1493,8 +1807,12 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
+      <c r="A28" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1521,8 +1839,12 @@
       <c r="Z28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
+      <c r="A29" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1549,8 +1871,12 @@
       <c r="Z29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
+      <c r="A30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1577,8 +1903,12 @@
       <c r="Z30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
+      <c r="A31" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -1605,8 +1935,12 @@
       <c r="Z31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="A32" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>57</v>
+      </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -1633,8 +1967,12 @@
       <c r="Z32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+      <c r="A33" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -1661,8 +1999,12 @@
       <c r="Z33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
+      <c r="A34" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -1689,8 +2031,12 @@
       <c r="Z34" s="2"/>
     </row>
     <row r="35">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
+      <c r="A35" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -1717,8 +2063,12 @@
       <c r="Z35" s="2"/>
     </row>
     <row r="36">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
+      <c r="A36" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -1745,8 +2095,12 @@
       <c r="Z36" s="2"/>
     </row>
     <row r="37">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
+      <c r="A37" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
@@ -1773,8 +2127,12 @@
       <c r="Z37" s="2"/>
     </row>
     <row r="38">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
+      <c r="A38" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
@@ -1801,8 +2159,12 @@
       <c r="Z38" s="2"/>
     </row>
     <row r="39">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
+      <c r="A39" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -1829,8 +2191,12 @@
       <c r="Z39" s="2"/>
     </row>
     <row r="40">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
+      <c r="A40" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
@@ -1857,8 +2223,12 @@
       <c r="Z40" s="2"/>
     </row>
     <row r="41">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
+      <c r="A41" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -1885,8 +2255,12 @@
       <c r="Z41" s="2"/>
     </row>
     <row r="42">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
+      <c r="A42" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -1913,8 +2287,12 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
+      <c r="A43" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -1941,8 +2319,12 @@
       <c r="Z43" s="2"/>
     </row>
     <row r="44">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
+      <c r="A44" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -1969,8 +2351,12 @@
       <c r="Z44" s="2"/>
     </row>
     <row r="45">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
+      <c r="A45" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -1997,8 +2383,12 @@
       <c r="Z45" s="2"/>
     </row>
     <row r="46">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
+      <c r="A46" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
@@ -2025,8 +2415,12 @@
       <c r="Z46" s="2"/>
     </row>
     <row r="47">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
+      <c r="A47" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
@@ -2053,8 +2447,12 @@
       <c r="Z47" s="2"/>
     </row>
     <row r="48">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
+      <c r="A48" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
@@ -2081,8 +2479,12 @@
       <c r="Z48" s="2"/>
     </row>
     <row r="49">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
+      <c r="A49" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
@@ -2109,8 +2511,12 @@
       <c r="Z49" s="2"/>
     </row>
     <row r="50">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
+      <c r="A50" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
@@ -2137,8 +2543,12 @@
       <c r="Z50" s="2"/>
     </row>
     <row r="51">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
+      <c r="A51" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
@@ -2165,8 +2575,12 @@
       <c r="Z51" s="2"/>
     </row>
     <row r="52">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
+      <c r="A52" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
@@ -2193,8 +2607,12 @@
       <c r="Z52" s="2"/>
     </row>
     <row r="53">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
+      <c r="A53" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>84</v>
+      </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
@@ -2221,8 +2639,12 @@
       <c r="Z53" s="2"/>
     </row>
     <row r="54">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
+      <c r="A54" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>86</v>
+      </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -2249,8 +2671,6 @@
       <c r="Z54" s="2"/>
     </row>
     <row r="55">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
@@ -2277,8 +2697,6 @@
       <c r="Z55" s="2"/>
     </row>
     <row r="56">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
@@ -2305,8 +2723,12 @@
       <c r="Z56" s="2"/>
     </row>
     <row r="57">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
+      <c r="A57" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B57" s="19" t="s">
+        <v>88</v>
+      </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
@@ -2333,8 +2755,12 @@
       <c r="Z57" s="2"/>
     </row>
     <row r="58">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
+      <c r="A58" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
@@ -2361,8 +2787,12 @@
       <c r="Z58" s="2"/>
     </row>
     <row r="59">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
+      <c r="A59" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -2389,8 +2819,12 @@
       <c r="Z59" s="2"/>
     </row>
     <row r="60">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
+      <c r="A60" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -2501,7 +2935,9 @@
       <c r="Z63" s="2"/>
     </row>
     <row r="64">
-      <c r="A64" s="2"/>
+      <c r="A64" s="3" t="s">
+        <v>94</v>
+      </c>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -2529,7 +2965,9 @@
       <c r="Z64" s="2"/>
     </row>
     <row r="65">
-      <c r="A65" s="2"/>
+      <c r="A65" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -2557,9 +2995,15 @@
       <c r="Z65" s="2"/>
     </row>
     <row r="66">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
+      <c r="A66" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>98</v>
+      </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
@@ -2585,8 +3029,12 @@
       <c r="Z66" s="2"/>
     </row>
     <row r="67">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
+      <c r="A67" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>100</v>
+      </c>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
@@ -28792,7 +29240,95 @@
       <c r="Y1002" s="2"/>
       <c r="Z1002" s="2"/>
     </row>
+    <row r="1003">
+      <c r="A1003" s="2"/>
+      <c r="B1003" s="2"/>
+      <c r="C1003" s="2"/>
+      <c r="D1003" s="2"/>
+      <c r="E1003" s="2"/>
+      <c r="F1003" s="2"/>
+      <c r="G1003" s="2"/>
+      <c r="H1003" s="2"/>
+      <c r="I1003" s="2"/>
+      <c r="J1003" s="2"/>
+      <c r="K1003" s="2"/>
+      <c r="L1003" s="2"/>
+      <c r="M1003" s="2"/>
+      <c r="N1003" s="2"/>
+      <c r="O1003" s="2"/>
+      <c r="P1003" s="2"/>
+      <c r="Q1003" s="2"/>
+      <c r="R1003" s="2"/>
+      <c r="S1003" s="2"/>
+      <c r="T1003" s="2"/>
+      <c r="U1003" s="2"/>
+      <c r="V1003" s="2"/>
+      <c r="W1003" s="2"/>
+      <c r="X1003" s="2"/>
+      <c r="Y1003" s="2"/>
+      <c r="Z1003" s="2"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="2"/>
+      <c r="B1004" s="2"/>
+      <c r="C1004" s="2"/>
+      <c r="D1004" s="2"/>
+      <c r="E1004" s="2"/>
+      <c r="F1004" s="2"/>
+      <c r="G1004" s="2"/>
+      <c r="H1004" s="2"/>
+      <c r="I1004" s="2"/>
+      <c r="J1004" s="2"/>
+      <c r="K1004" s="2"/>
+      <c r="L1004" s="2"/>
+      <c r="M1004" s="2"/>
+      <c r="N1004" s="2"/>
+      <c r="O1004" s="2"/>
+      <c r="P1004" s="2"/>
+      <c r="Q1004" s="2"/>
+      <c r="R1004" s="2"/>
+      <c r="S1004" s="2"/>
+      <c r="T1004" s="2"/>
+      <c r="U1004" s="2"/>
+      <c r="V1004" s="2"/>
+      <c r="W1004" s="2"/>
+      <c r="X1004" s="2"/>
+      <c r="Y1004" s="2"/>
+      <c r="Z1004" s="2"/>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="2"/>
+      <c r="B1005" s="2"/>
+      <c r="C1005" s="2"/>
+      <c r="D1005" s="2"/>
+      <c r="E1005" s="2"/>
+      <c r="F1005" s="2"/>
+      <c r="G1005" s="2"/>
+      <c r="H1005" s="2"/>
+      <c r="I1005" s="2"/>
+      <c r="J1005" s="2"/>
+      <c r="K1005" s="2"/>
+      <c r="L1005" s="2"/>
+      <c r="M1005" s="2"/>
+      <c r="N1005" s="2"/>
+      <c r="O1005" s="2"/>
+      <c r="P1005" s="2"/>
+      <c r="Q1005" s="2"/>
+      <c r="R1005" s="2"/>
+      <c r="S1005" s="2"/>
+      <c r="T1005" s="2"/>
+      <c r="U1005" s="2"/>
+      <c r="V1005" s="2"/>
+      <c r="W1005" s="2"/>
+      <c r="X1005" s="2"/>
+      <c r="Y1005" s="2"/>
+      <c r="Z1005" s="2"/>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B54:B56"/>
+  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -28810,7 +29346,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
@@ -28818,75 +29354,91 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>46</v>
+      <c r="B2" s="20" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>48</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>50</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="s">
-        <v>51</v>
+      <c r="A5" s="21" t="s">
+        <v>108</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>52</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="s">
-        <v>53</v>
+      <c r="A6" s="21" t="s">
+        <v>110</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>55</v>
+        <v>112</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>56</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>57</v>
+        <v>114</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>58</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>59</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>60</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
       <c r="B11" s="2"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>122</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -28906,6 +29458,73 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="s">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="A1"/>
+  </hyperlinks>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="24.88"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="28.25"/>
     <col customWidth="1" min="2" max="2" width="45.0"/>
@@ -28913,7 +29532,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -28945,7 +29564,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -28974,11 +29593,11 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="s">
-        <v>63</v>
+      <c r="A3" s="27" t="s">
+        <v>132</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>64</v>
+        <v>133</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -29006,11 +29625,11 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="s">
-        <v>51</v>
+      <c r="A4" s="21" t="s">
+        <v>108</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>52</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -29038,11 +29657,11 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="s">
-        <v>53</v>
+      <c r="A5" s="21" t="s">
+        <v>110</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -29071,10 +29690,10 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>55</v>
+        <v>112</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>56</v>
+        <v>113</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -29103,10 +29722,10 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>57</v>
+        <v>114</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>58</v>
+        <v>115</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -29135,7 +29754,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>59</v>
+        <v>116</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -29164,7 +29783,7 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>60</v>
+        <v>117</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -29193,7 +29812,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -56950,7 +57569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -56962,7 +57581,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
@@ -56970,10 +57589,10 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>65</v>
+        <v>134</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>66</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>